<commit_message>
In this commit, the current trend slope was estimated using a 10 year-interval window rather than the usual 9 year-interval window for all masks and states. That is, the current trend start year was set to 2015 instead of … …2016. As a consequence, the SoIB main file, trends file and other associated outputs were also re-generated. The website xlsx file has also been generated.
</commit_message>
<xml_diff>
--- a/01_analyses_mask-ONEland/results/SoIB_summaries.xlsx
+++ b/01_analyses_mask-ONEland/results/SoIB_summaries.xlsx
@@ -11,11 +11,136 @@
     <sheet name="Range Status" sheetId="2" r:id="rId2"/>
     <sheet name="Priority Status" sheetId="3" r:id="rId3"/>
     <sheet name="Species qualification" sheetId="4" r:id="rId4"/>
-    <sheet name="Interannual update - High Pri" sheetId="5" r:id="rId5"/>
-    <sheet name="Major update - High Priority " sheetId="6" r:id="rId6"/>
+    <sheet name="Interannual update - High Prior" sheetId="5" r:id="rId5"/>
+    <sheet name="Major update - High Priority br" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+  <si>
+    <t>Trend Status</t>
+  </si>
+  <si>
+    <t>Long-term species (no.)</t>
+  </si>
+  <si>
+    <t>Current species (no.)</t>
+  </si>
+  <si>
+    <t>Long-term species conclusive (perc.)</t>
+  </si>
+  <si>
+    <t>Current species conclusive (perc.)</t>
+  </si>
+  <si>
+    <t>Rapid Decline</t>
+  </si>
+  <si>
+    <t>Decline</t>
+  </si>
+  <si>
+    <t>Stable</t>
+  </si>
+  <si>
+    <t>Increase</t>
+  </si>
+  <si>
+    <t>Rapid Increase</t>
+  </si>
+  <si>
+    <t>Trend Inconclusive</t>
+  </si>
+  <si>
+    <t>Insufficient Data</t>
+  </si>
+  <si>
+    <t>Range Status</t>
+  </si>
+  <si>
+    <t>Species (no.)</t>
+  </si>
+  <si>
+    <t>Species (perc.)</t>
+  </si>
+  <si>
+    <t>Historical</t>
+  </si>
+  <si>
+    <t>Very Restricted</t>
+  </si>
+  <si>
+    <t>Restricted</t>
+  </si>
+  <si>
+    <t>Moderate</t>
+  </si>
+  <si>
+    <t>Large</t>
+  </si>
+  <si>
+    <t>Very Large</t>
+  </si>
+  <si>
+    <t>Priority Status</t>
+  </si>
+  <si>
+    <t>No. of species</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>No. of species in:</t>
+  </si>
+  <si>
+    <t>Selected for analysis</t>
+  </si>
+  <si>
+    <t>With conclusive trends</t>
+  </si>
+  <si>
+    <t>SoIB Assessment</t>
+  </si>
+  <si>
+    <t>Long-term Analysis</t>
+  </si>
+  <si>
+    <t>Current Analysis</t>
+  </si>
+  <si>
+    <t>Range Analysis</t>
+  </si>
+  <si>
+    <t>Break-up</t>
+  </si>
+  <si>
+    <t>High Species (no.)</t>
+  </si>
+  <si>
+    <t>High Species (perc.)</t>
+  </si>
+  <si>
+    <t>New High Species (no.)</t>
+  </si>
+  <si>
+    <t>New High Species (perc.)</t>
+  </si>
+  <si>
+    <t>Trend New</t>
+  </si>
+  <si>
+    <t>Trend Different</t>
+  </si>
+  <si>
+    <t>IUCN</t>
+  </si>
+</sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -359,38 +484,26 @@
   <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Trend Status</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Long-term species (no.)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Current species (no.)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Long-term species conclusive (perc.)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>Current species conclusive (perc.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Rapid Decline</t>
-        </is>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>5</v>
       </c>
       <c r="B2">
         <v>11</v>
@@ -402,71 +515,63 @@
         <v>45.8</v>
       </c>
       <c r="E2">
-        <v>10.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Decline</t>
-        </is>
+        <v>9.1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>6</v>
       </c>
       <c r="B3">
         <v>8</v>
       </c>
       <c r="C3">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="D3">
         <v>33.3</v>
       </c>
       <c r="E3">
-        <v>47.4</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+        <v>54.5</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>7</v>
       </c>
       <c r="B4">
         <v>3</v>
       </c>
       <c r="C4">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D4">
         <v>12.5</v>
       </c>
       <c r="E4">
-        <v>42.1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Increase</t>
-        </is>
+        <v>31.8</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5">
+      <c r="A5" t="s">
+        <v>8</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D5">
         <v>4.2</v>
       </c>
       <c r="E5">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Rapid Increase</t>
-        </is>
+        <v>4.5</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5">
+      <c r="A6" t="s">
+        <v>9</v>
       </c>
       <c r="B6">
         <v>1</v>
@@ -481,24 +586,20 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Trend Inconclusive</t>
-        </is>
+    <row r="7" spans="1:5">
+      <c r="A7" t="s">
+        <v>10</v>
       </c>
       <c r="B7">
         <v>11</v>
       </c>
       <c r="C7">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Insufficient Data</t>
-        </is>
+        <v>28</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5">
+      <c r="A8" t="s">
+        <v>11</v>
       </c>
       <c r="B8">
         <v>82</v>
@@ -517,78 +618,60 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Range Status</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Species (no.)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Species (perc.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Historical</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>15</v>
       </c>
       <c r="B2">
         <v>0</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Very Restricted</t>
-        </is>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>16</v>
       </c>
       <c r="B3">
         <v>0</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Restricted</t>
-        </is>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>17</v>
       </c>
       <c r="B4">
         <v>0</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>18</v>
       </c>
       <c r="B5">
         <v>0</v>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Large</t>
-        </is>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>19</v>
       </c>
       <c r="B6">
         <v>0</v>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Very Large</t>
-        </is>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>20</v>
       </c>
       <c r="B7">
         <v>0</v>
@@ -604,46 +687,36 @@
   <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Priority Status</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>No. of species</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
+    <row r="1" spans="1:2" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>23</v>
       </c>
       <c r="B2">
-        <v>103</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Moderate</t>
-        </is>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>18</v>
       </c>
       <c r="B3">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Low</t>
-        </is>
+        <v>392</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>24</v>
       </c>
       <c r="B4">
-        <v>441</v>
+        <v>433</v>
       </c>
     </row>
   </sheetData>
@@ -656,38 +729,28 @@
   <dimension ref="A1:C5"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>No. of species in:</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Selected for analysis</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>With conclusive trends</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>SoIB Assessment</t>
-        </is>
+    <row r="1" spans="1:3" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>28</v>
       </c>
       <c r="B2">
         <v>117</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Long-term Analysis</t>
-        </is>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>29</v>
       </c>
       <c r="B3">
         <v>35</v>
@@ -696,24 +759,20 @@
         <v>24</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Current Analysis</t>
-        </is>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>30</v>
       </c>
       <c r="B4">
         <v>50</v>
       </c>
       <c r="C4">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>Range Analysis</t>
-        </is>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>31</v>
       </c>
       <c r="B5">
         <v>0</v>
@@ -729,88 +788,66 @@
   <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Break-up</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>High Species (no.)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>High Species (perc.)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>New High Species (no.)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>New High Species (perc.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Trend New</t>
-        </is>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>37</v>
       </c>
       <c r="B2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C2">
-        <v>83.5</v>
+        <v>84</v>
       </c>
       <c r="D2">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="E2">
-        <v>96.59999999999999</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Trend Different</t>
-        </is>
+        <v>96.7</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>38</v>
       </c>
       <c r="B3">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C3">
-        <v>4.9</v>
-      </c>
-      <c r="D3">
-        <v>1</v>
-      </c>
-      <c r="E3">
-        <v>1.1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>IUCN</t>
-        </is>
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5">
+      <c r="A4" t="s">
+        <v>39</v>
       </c>
       <c r="B4">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C4">
-        <v>11.7</v>
+        <v>12.3</v>
       </c>
       <c r="D4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E4">
-        <v>2.2</v>
+        <v>3.3</v>
       </c>
     </row>
   </sheetData>
@@ -823,38 +860,26 @@
   <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" s="1" customFormat="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Break-up</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>High Species (no.)</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>High Species (perc.)</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>New High Species (no.)</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>New High Species (perc.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Trend New</t>
-        </is>
+    <row r="1" spans="1:5" s="1" customFormat="1">
+      <c r="A1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5">
+      <c r="A2" t="s">
+        <v>37</v>
       </c>
       <c r="B2">
         <v>12</v>
@@ -869,11 +894,9 @@
         <v>48</v>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>IUCN</t>
-        </is>
+    <row r="3" spans="1:5">
+      <c r="A3" t="s">
+        <v>39</v>
       </c>
       <c r="B3">
         <v>13</v>

</xml_diff>